<commit_message>
Add nutrition set selection (STTM row 14) and rule R23
select_nutrition_set picks one set per product: as_sold, preferred basis
(100ml for ml products, else 100g), then manufacturer > packaging > estimate,
with a fallback to the other basis. STTM: add R23_assumed_basis, extend
row 14 with the fallback, correct the R01 evidence note (line 642 has an
empty code).
</commit_message>
<xml_diff>
--- a/docs/sttm.xlsx
+++ b/docs/sttm.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4" customWidth="1" style="9" min="1" max="1"/>
@@ -631,7 +631,7 @@
       </c>
       <c r="L2" s="12" t="inlineStr">
         <is>
-          <t>100% present in profile</t>
+          <t>7,628 of 7,629 present; line 642 of the delta file has an empty code (checked 8 Oct 2026)</t>
         </is>
       </c>
     </row>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>select ONE set: preparation = as_sold; per = 100g (100ml if quantity_unit = ml); precedence manufacturer &gt; packaging &gt; estimate</t>
+          <t>select ONE set: preparation = as_sold; per = 100g (100ml if quantity_unit = ml); precedence manufacturer &gt; packaging &gt; estimate; basis fallback: if no set matches the preferred basis, use the other one (100g for ml products, 100ml for products whose unit is not ml) and flag R23</t>
         </is>
       </c>
       <c r="F15" s="12" t="inlineStr">
@@ -2372,6 +2372,66 @@
       <c r="L31" s="12" t="inlineStr">
         <is>
           <t>lineage: which file, when</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="23.85" customHeight="1" s="10">
+      <c r="A32" s="12" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>nutrition.input_sets[]</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>nutrition_basis</t>
+        </is>
+      </c>
+      <c r="D32" s="12" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E32" s="12" t="inlineStr">
+        <is>
+          <t>as row 14 (basis fallback)</t>
+        </is>
+      </c>
+      <c r="F32" s="12" t="inlineStr">
+        <is>
+          <t>selected set's basis equals the preferred basis (100ml for ml products, 100g otherwise)</t>
+        </is>
+      </c>
+      <c r="G32" s="12" t="inlineStr">
+        <is>
+          <t>R23_assumed_basis</t>
+        </is>
+      </c>
+      <c r="H32" s="12" t="inlineStr">
+        <is>
+          <t>validity</t>
+        </is>
+      </c>
+      <c r="I32" s="14" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="J32" s="12" t="inlineStr">
+        <is>
+          <t>measure only</t>
+        </is>
+      </c>
+      <c r="K32" s="12" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L32" s="12" t="inlineStr">
+        <is>
+          <t>Added 8 Oct 2026. Only for liquids with density near 1 is 100g ≈ 100ml. In the 7 Oct delta file, 142 ml products have only a per-100g set (98 with kcal). 74 products with both sets: median kcal(100ml)/kcal(100g) = 1.0, range 0.2–3.55 (extremes probably data errors). Not converted; the basis actually used is stored in nutrition_basis.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Set R02 to optional until failure sample is reviewed
</commit_message>
<xml_diff>
--- a/docs/sttm.xlsx
+++ b/docs/sttm.xlsx
@@ -676,12 +676,12 @@
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
-          <t>important</t>
+          <t>optional</t>
         </is>
       </c>
       <c r="J3" s="12" t="inlineStr">
         <is>
-          <t>keep row, flag</t>
+          <t>measure only</t>
         </is>
       </c>
       <c r="K3" s="12" t="inlineStr">
@@ -691,7 +691,7 @@
       </c>
       <c r="L3" s="12" t="inlineStr">
         <is>
-          <t>Checked 5 Oct: no GTIN check-digit validation in OFF's DataQuality.pm, DataQualityCommon.pm or DataQualityFood.pm (only GS1-prefix pattern checks), so this is our own rule, not an OFF duplicate. No OFF flag to benchmark against. Not checked outside those three files.</t>
+          <t>Checked 5 Oct: no GTIN check-digit validation in OFF's DataQuality.pm, DataQualityCommon.pm or DataQualityFood.pm (only GS1-prefix pattern checks), so this is our own rule, not an OFF duplicate. No OFF flag to benchmark against. Not checked outside those three files. Severity set to optional on 10 Oct 2026: a failing code is not a valid GTIN, but not proven to be an error (OFF may hold non-GTIN codes; unverified). Report by failure type (non_digit, bad_length, bad_check_digit). Promote to important if a 20-row sample of failures shows mostly typos.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add rules R15 to R19, record R12 R14 R20 as not implemented
</commit_message>
<xml_diff>
--- a/docs/sttm.xlsx
+++ b/docs/sttm.xlsx
@@ -1471,7 +1471,7 @@
       </c>
       <c r="L16" s="12" t="inlineStr">
         <is>
-          <t>packaging·as_sold·serving = 1,884 sets</t>
+          <t>packaging·as_sold·serving = 1,884 sets Status 11 Oct 2026: designed, not implemented in v1. Staging keeps only the chosen nutrition set, so serving-only products cannot be told apart from other 'no usable set' cases (R11 includes them). Needs raw set information.</t>
         </is>
       </c>
     </row>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="L18" s="12" t="inlineStr">
         <is>
-          <t>own rule; rare (manufacturer data scarce)</t>
+          <t>own rule; rare (manufacturer data scarce) Status 11 Oct 2026: designed, not implemented in v1. Needs both the manufacturer and the packaging set, staging keeps only one.</t>
         </is>
       </c>
     </row>
@@ -1651,7 +1651,7 @@
       </c>
       <c r="L19" s="12" t="inlineStr">
         <is>
-          <t>sample max 851 (plausible)</t>
+          <t>sample max 851 (plausible) Implemented 11 Oct 2026. Threshold: energy_kcal &gt; 935 per 100g/ml (OFF flags 3,911 kJ; 3,911 / 4.184 = 934.8 kcal) or negative. Delta file: 12 failures, 4 from editor municorn-calorie-counter-app. At least 5 of the 12 values equal a per-serving number divided by a round serving size times 100 (e.g. 64 kcal / 3 g = 2,133); inferred from the arithmetic, not checked in the raw records.</t>
         </is>
       </c>
     </row>
@@ -1711,7 +1711,7 @@
       </c>
       <c r="L20" s="12" t="inlineStr">
         <is>
-          <t>zero alone is NOT an error (oil has 0 sugar)</t>
+          <t>zero alone is NOT an error (oil has 0 sugar) Implemented 11 Oct 2026. Threshold: fat, saturated fat, carbs, sugars, protein or fibre outside 0 to 105 g, or fat + carbs + protein &gt; 105 g (OFF uses 105 g; its sum also includes salt, left out here so a salt error appears once, under R17). Delta file: 14 failures.</t>
         </is>
       </c>
     </row>
@@ -1771,7 +1771,7 @@
       </c>
       <c r="L21" s="12" t="inlineStr">
         <is>
-          <t>sample max 720 g / 100 g</t>
+          <t>sample max 720 g / 100 g Implemented 11 Oct 2026. Threshold: salt_g &gt; 105. Delta file: 5 failures, catches 5 of 7 known outliers; a sodium x1000 error whose salt lands between 25 and 105 g passes a ceiling check. OFF has no dedicated salt-too-high tag. OFF's salt-does-not-match-sodium flag (93 products in the delta file) is not reproduced: staging keeps only the final salt_g.</t>
         </is>
       </c>
     </row>
@@ -1831,7 +1831,7 @@
       </c>
       <c r="L22" s="12" t="inlineStr">
         <is>
-          <t>Checked 5 Oct: partly overlaps OFF. OFF flags energy when computed energy is outside stated x 0.7 - 5 .. stated x 1.3 + 5 (tag family '...energy-value-in-&lt;unit&gt;-does-not-match-value-computed-from-other-nutrients'), which also catches most 0-vs-macros cases. Kept as our own simple, explainable rule; benchmark its hits against OFF's tags.</t>
+          <t>Checked 5 Oct: partly overlaps OFF. OFF flags energy when computed energy is outside stated x 0.7 - 5 .. stated x 1.3 + 5 (tag family '...energy-value-in-&lt;unit&gt;-does-not-match-value-computed-from-other-nutrients'), which also catches most 0-vs-macros cases. Kept as our own simple, explainable rule; benchmark its hits against OFF's tags. Implemented 11 Oct 2026. Computed kcal = 9 fat + 4 carbs + 4 protein + 2 fibre; failure if outside 0.7 x stated - 5 to 1.3 x stated + 5 (OFF's strong-mismatch band), only when energy &gt; 13 kcal and fat, carbs and protein are present. The formula is our approximation (no alcohol, polyols or organic acids). Delta file: 119 failures. Against OFF's own flag on the same chosen set: 93 flagged by both, 26 only by us, 23 only by OFF; reasons for the differences not checked.</t>
         </is>
       </c>
     </row>
@@ -1891,7 +1891,7 @@
       </c>
       <c r="L23" s="12" t="inlineStr">
         <is>
-          <t>Checked 5 Oct: saturated-fat &gt; fat is identical to OFF's check. OFF's carbs check is sugars + starch &gt; carbohydrates (stricter than sugars alone), with tolerance 0.01 g below 10 g and 0.1 g from 10 g up. Decide at coding time whether to add starch and a tolerance; without one, rounding causes false flags. Benchmark vs OFF tags 'saturated-fat-greater-than-fat' and 'sugars-plus-starch-greater-than-carbohydrates'.</t>
+          <t>Checked 5 Oct: saturated-fat &gt; fat is identical to OFF's check. OFF's carbs check is sugars + starch &gt; carbohydrates (stricter than sugars alone), with tolerance 0.01 g below 10 g and 0.1 g from 10 g up. Decide at coding time whether to add starch and a tolerance; without one, rounding causes false flags. Benchmark vs OFF tags 'saturated-fat-greater-than-fat' and 'sugars-plus-starch-greater-than-carbohydrates'. Implemented 11 Oct 2026. Sugars &gt; carbs, or saturated fat &gt; fat, with OFF's tolerance (0.01 g, 0.1 g when the total is 10 g or more). Delta file: 12 failures. No starch column in staging, so OFF's sugars + starch &gt; carbs check is only approximated.</t>
         </is>
       </c>
     </row>
@@ -1951,7 +1951,7 @@
       </c>
       <c r="L24" s="12" t="inlineStr">
         <is>
-          <t>pattern seen in profiled record</t>
+          <t>pattern seen in profiled record Status 11 Oct 2026: designed, not implemented in v1. Micronutrients are not loaded into staging.</t>
         </is>
       </c>
     </row>

</xml_diff>